<commit_message>
data(realSuite): regenerate input.xlsx with grouped schools included
Re-run the extract phase to regenerate all 29 test case input.xlsx files using
the fixed extract_schools_from_structured() function. This now includes schools
that share a pickup point (grouped schools via forward-fill from Dettaglio
Completo). For example, Padel case goes from 8 to 10 schools (gains IS GUETTI
and IS FILZI ROVERETO).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/realSuite/Piani-viaggio_Padel_10-dic-25_def2_con-VETTORE/input.xlsx
+++ b/tests/realSuite/Piani-viaggio_Padel_10-dic-25_def2_con-VETTORE/input.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -511,45 +511,75 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IS FLORIANI RIVA DEL GARDA</t>
+          <t>IS FILZI ROVERETO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Riva del Garda, V.le dei Tigli 43</t>
+          <t>Rovereto, P.le Orsi</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>IS M. MARTINI MEZZOLOMBARDO</t>
+          <t>IS FLORIANI RIVA DEL GARDA</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Mezzolombardo, Via Perlasca 4</t>
+          <t>Riva del Garda, V.le dei Tigli 43</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>IS GUETTI</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tione, Via Durone 53 – fermata davanti alla scuola I.I.L. Guetti</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>IS M. MARTINI MEZZOLOMBARDO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Mezzolombardo, Via Perlasca 4</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>IS MAFFEI RIVA DEL GARDA</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>Riva del Garda, V.le Martiri, fermata autobus</t>
         </is>
       </c>
-      <c r="C9" t="n">
+      <c r="C11" t="n">
         <v>9</v>
       </c>
     </row>

</xml_diff>